<commit_message>
Ajustes de exportación de datos y mejoras de rendimiento
</commit_message>
<xml_diff>
--- a/Documentación/brecha API.xlsx
+++ b/Documentación/brecha API.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD494406-BADC-4B74-AA30-7DEC985F7CDE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A248FE-4EBC-40B9-BEE2-78A9130AF128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Vida - Emision" sheetId="3" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="90">
   <si>
     <t>Módulo / Sección</t>
   </si>
@@ -287,7 +287,72 @@
     <t>Manejar como grupal</t>
   </si>
   <si>
-    <t>Plan UNICA</t>
+    <t>Solo se renueva y se cancela</t>
+  </si>
+  <si>
+    <t>Plan 10</t>
+  </si>
+  <si>
+    <t>En renovación solo se valida un % del pendiente y si no es mayor al 20% se renueva de manera automática</t>
+  </si>
+  <si>
+    <t>Endoso de beneficiarios
+Se manejan descuentos/recargos de manera rara, pero se usan</t>
+  </si>
+  <si>
+    <t>Documentos: poliza plan 10, ofeta, listas de beneficiarios (2), recibo</t>
+  </si>
+  <si>
+    <t>PLAN20</t>
+  </si>
+  <si>
+    <t>PLAN30</t>
+  </si>
+  <si>
+    <t>PLAN50</t>
+  </si>
+  <si>
+    <t>No se usan</t>
+  </si>
+  <si>
+    <t>Cambio de edad en renovación afecta prima
+Para efectos de renovaciones no mantener recargos/descuentos
+Vigencia anual</t>
+  </si>
+  <si>
+    <t>PLAN UNICA clasica/platinum</t>
+  </si>
+  <si>
+    <t>Declarativa mensual
+Vigencia mensual
+Hay un reporte del banco
+Alguna pólizas quedan vencidas (no se renuevan)
+Se colocan como no renovadas (una a una)
+No existe interfaz de renovación por parte del banco</t>
+  </si>
+  <si>
+    <t>Generales</t>
+  </si>
+  <si>
+    <t>Documento de endoso para cambio de beneficiarios (todos los productos)</t>
+  </si>
+  <si>
+    <t>Renovación
+Cancelación
+Cambio de beneficario
+Recargos/descuentos</t>
+  </si>
+  <si>
+    <t>Forma de pago cuenta a cuenta
+Hacen cambios de plan cuando está creada la oferta
+Pago unico mensual pagado por el banco</t>
+  </si>
+  <si>
+    <t>Documentos: poliza (Plan Mujer), oferta, recibo, beneficiarios</t>
+  </si>
+  <si>
+    <t>Se emiten nuevas
+Ver edades de adminisión y renovación para todos los planes</t>
   </si>
 </sst>
 </file>
@@ -680,7 +745,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:H12"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -860,6 +925,67 @@
       </c>
       <c r="H12" s="6" t="s">
         <v>71</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B14" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B15" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B18" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H18" s="6" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B19" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B20" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H20" s="6" t="s">
+        <v>88</v>
       </c>
     </row>
   </sheetData>
@@ -934,7 +1060,7 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>67</v>
@@ -950,7 +1076,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="23.85546875" style="4" bestFit="1" customWidth="1"/>
@@ -1069,6 +1195,67 @@
       </c>
       <c r="H7" s="1" t="s">
         <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B8" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B9" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B10" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B11" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="B12" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="B13" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="B14" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustes fusión de pagos
</commit_message>
<xml_diff>
--- a/Documentación/brecha API.xlsx
+++ b/Documentación/brecha API.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48A248FE-4EBC-40B9-BEE2-78A9130AF128}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B77FCE-5FE7-4422-AFD9-8ACF5A88A602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="98">
   <si>
     <t>Módulo / Sección</t>
   </si>
@@ -343,16 +343,42 @@
 Recargos/descuentos</t>
   </si>
   <si>
-    <t>Forma de pago cuenta a cuenta
+    <t>No</t>
+  </si>
+  <si>
+    <t>Ninguna</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Validar </t>
+  </si>
+  <si>
+    <t>Pendiente para brecha de reclamos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Configurar catálogos de sis9 y validar </t>
+  </si>
+  <si>
+    <t>Existe</t>
+  </si>
+  <si>
+    <t>Validar funcionalidad</t>
+  </si>
+  <si>
+    <t>Validar y configurar</t>
+  </si>
+  <si>
+    <t>Se emiten nuevas
+Ver edades de adminisión y renovación para todos los planes
+Forma de pago cuenta a cuenta
 Hacen cambios de plan cuando está creada la oferta
-Pago unico mensual pagado por el banco</t>
-  </si>
-  <si>
-    <t>Documentos: poliza (Plan Mujer), oferta, recibo, beneficiarios</t>
-  </si>
-  <si>
-    <t>Se emiten nuevas
-Ver edades de adminisión y renovación para todos los planes</t>
+Pago unico mensual pagado por el banco
+Documentos: poliza (Plan Mujer), oferta, recibo, beneficiarios</t>
+  </si>
+  <si>
+    <t>Configurar y desarrollar</t>
+  </si>
+  <si>
+    <t>Configurar y Desarrollar</t>
   </si>
 </sst>
 </file>
@@ -419,14 +445,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -745,7 +771,7 @@
   <sheetPr>
     <tabColor rgb="FFFF0000"/>
   </sheetPr>
-  <dimension ref="A1:H20"/>
+  <dimension ref="A1:H19"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" style="4" bestFit="1" customWidth="1"/>
@@ -835,6 +861,21 @@
       <c r="B4" s="4" t="s">
         <v>32</v>
       </c>
+      <c r="C4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>93</v>
+      </c>
       <c r="H4" s="6" t="s">
         <v>33</v>
       </c>
@@ -846,6 +887,21 @@
       <c r="B5" s="4" t="s">
         <v>39</v>
       </c>
+      <c r="C5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>93</v>
+      </c>
       <c r="H5" s="6" t="s">
         <v>40</v>
       </c>
@@ -857,6 +913,21 @@
       <c r="B6" s="4" t="s">
         <v>41</v>
       </c>
+      <c r="C6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="H6" s="6" t="s">
         <v>42</v>
       </c>
@@ -868,6 +939,21 @@
       <c r="B7" s="4" t="s">
         <v>43</v>
       </c>
+      <c r="C7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="H7" s="6" t="s">
         <v>48</v>
       </c>
@@ -879,6 +965,21 @@
       <c r="B8" s="4" t="s">
         <v>44</v>
       </c>
+      <c r="C8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>88</v>
+      </c>
       <c r="H8" s="6" t="s">
         <v>45</v>
       </c>
@@ -890,6 +991,21 @@
       <c r="B9" s="4" t="s">
         <v>53</v>
       </c>
+      <c r="C9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="H9" s="6" t="s">
         <v>51</v>
       </c>
@@ -901,6 +1017,21 @@
       <c r="B10" s="4" t="s">
         <v>53</v>
       </c>
+      <c r="C10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="H10" s="6" t="s">
         <v>54</v>
       </c>
@@ -912,6 +1043,21 @@
       <c r="B11" s="4" t="s">
         <v>61</v>
       </c>
+      <c r="C11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="H11" s="6" t="s">
         <v>65</v>
       </c>
@@ -923,70 +1069,160 @@
       <c r="B12" s="4" t="s">
         <v>70</v>
       </c>
+      <c r="C12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>94</v>
+      </c>
       <c r="H12" s="6" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="B13" s="4" t="s">
         <v>73</v>
       </c>
+      <c r="C13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="B14" s="4" t="s">
-        <v>73</v>
+        <v>77</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>88</v>
       </c>
       <c r="H14" s="6" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="B15" s="4" t="s">
-        <v>77</v>
+        <v>78</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>88</v>
       </c>
       <c r="H15" s="6" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="B16" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F16" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>88</v>
       </c>
       <c r="H16" s="6" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="B17" s="4" t="s">
-        <v>79</v>
+        <v>82</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F17" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G17" s="4" t="s">
+        <v>94</v>
       </c>
       <c r="H17" s="6" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="18" spans="2:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="B18" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="19" spans="2:8" ht="45" x14ac:dyDescent="0.25">
-      <c r="B19" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="H19" s="6" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
-      <c r="B20" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>88</v>
-      </c>
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E18" s="2"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="E19" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1004,7 +1240,7 @@
     <col min="1" max="1" width="16.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="22.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="11.42578125" style="4"/>
-    <col min="7" max="7" width="13.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="120.5703125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1027,7 +1263,7 @@
       <c r="F2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="7" t="s">
         <v>6</v>
       </c>
       <c r="H2" s="5" t="s">
@@ -1038,6 +1274,21 @@
       <c r="B3" s="4" t="s">
         <v>46</v>
       </c>
+      <c r="C3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="H3" s="6" t="s">
         <v>47</v>
       </c>
@@ -1046,6 +1297,21 @@
       <c r="B4" s="4" t="s">
         <v>50</v>
       </c>
+      <c r="C4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H4" s="6" t="s">
         <v>49</v>
       </c>
@@ -1054,6 +1320,21 @@
       <c r="B5" s="4" t="s">
         <v>61</v>
       </c>
+      <c r="C5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H5" s="6" t="s">
         <v>68</v>
       </c>
@@ -1061,6 +1342,21 @@
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>73</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="H6" s="6" t="s">
         <v>67</v>
@@ -1082,7 +1378,7 @@
     <col min="1" max="1" width="23.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="25.7109375" style="3" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="5.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.42578125" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.42578125" style="3" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="121" style="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1165,94 +1461,286 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B4" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="C4" s="4"/>
+      <c r="C4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H4" s="1" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B5" s="3" t="s">
         <v>63</v>
       </c>
+      <c r="C5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H5" s="1" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B6" s="4" t="s">
         <v>61</v>
       </c>
+      <c r="C6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>11</v>
+      </c>
       <c r="H6" s="1" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B7" s="3" t="s">
         <v>52</v>
       </c>
+      <c r="C7" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>97</v>
+      </c>
       <c r="H7" s="1" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B8" s="4" t="s">
         <v>73</v>
       </c>
+      <c r="C8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H8" s="1" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B9" s="4" t="s">
         <v>73</v>
       </c>
+      <c r="C9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>88</v>
+      </c>
       <c r="H9" s="1" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B10" s="4" t="s">
         <v>73</v>
       </c>
+      <c r="C10" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>11</v>
+      </c>
       <c r="H10" s="1" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B11" s="4" t="s">
         <v>73</v>
       </c>
+      <c r="C11" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G11" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H11" s="1" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="90" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B12" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="C12" s="4"/>
-      <c r="D12" s="4"/>
-      <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
+      <c r="C12" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H12" s="6" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B13" s="4" t="s">
         <v>84</v>
       </c>
+      <c r="C13" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G13" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="H13" s="1" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
+        <v>19</v>
+      </c>
       <c r="B14" s="4" t="s">
         <v>82</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G14" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="H14" s="1" t="s">
         <v>86</v>
@@ -1274,7 +1762,9 @@
   <cols>
     <col min="1" max="1" width="16.5703125" style="4" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="31.5703125" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="89.85546875" customWidth="1"/>
+    <col min="6" max="6" width="11.42578125" style="4"/>
+    <col min="7" max="7" width="11.42578125" style="3"/>
+    <col min="8" max="8" width="89.85546875" style="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -1296,10 +1786,10 @@
       <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="8" t="s">
         <v>7</v>
       </c>
     </row>
@@ -1319,10 +1809,10 @@
       <c r="E2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" s="10" t="s">
+      <c r="F2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="3" t="s">
         <v>18</v>
       </c>
       <c r="H2" s="9" t="s">
@@ -1345,7 +1835,13 @@
       <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H3" s="1" t="s">
+      <c r="F3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="H3" s="9" t="s">
         <v>37</v>
       </c>
     </row>
@@ -1365,7 +1861,13 @@
       <c r="E4" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H4" s="1" t="s">
+      <c r="F4" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H4" s="9" t="s">
         <v>36</v>
       </c>
     </row>
@@ -1385,11 +1887,17 @@
       <c r="E5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="H5" t="s">
+      <c r="F5" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="H5" s="10" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
         <v>20</v>
       </c>
@@ -1405,7 +1913,13 @@
       <c r="E6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H6" t="s">
+      <c r="F6" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="H6" s="10" t="s">
         <v>27</v>
       </c>
     </row>
@@ -1420,12 +1934,18 @@
         <v>8</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="H7" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G7" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="H7" s="9" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1445,7 +1965,13 @@
       <c r="E8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H8" t="s">
+      <c r="F8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="10" t="s">
         <v>30</v>
       </c>
     </row>
@@ -1456,19 +1982,32 @@
       <c r="B9" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="H9" s="1" t="s">
+      <c r="C9" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="G9" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" s="9" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="H10" s="1"/>
+      <c r="H10" s="9"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="C12" s="4"/>
       <c r="D12" s="4"/>
       <c r="E12" s="4"/>
-      <c r="F12" s="4"/>
-      <c r="G12" s="4"/>
       <c r="H12" s="6"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Ajustes pago de reclamos
</commit_message>
<xml_diff>
--- a/Documentación/brecha API.xlsx
+++ b/Documentación/brecha API.xlsx
@@ -8,15 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Proyectos\Global\Documentación\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{28B77FCE-5FE7-4422-AFD9-8ACF5A88A602}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0E78A4D-387B-43C9-9D11-4089F1679CD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="3" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{55631BAB-3F43-4C4D-BEDF-0998D0E484F9}"/>
   </bookViews>
   <sheets>
     <sheet name="Vida - Emision" sheetId="3" r:id="rId1"/>
     <sheet name="Vida - Reaseguro" sheetId="4" r:id="rId2"/>
     <sheet name="Vida-Endoso" sheetId="6" r:id="rId3"/>
     <sheet name="Vida - Siniestro" sheetId="7" r:id="rId4"/>
+    <sheet name="Vida - Contabilidad" sheetId="8" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="352" uniqueCount="98">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="104">
   <si>
     <t>Módulo / Sección</t>
   </si>
@@ -379,6 +380,24 @@
   </si>
   <si>
     <t>Configurar y Desarrollar</t>
+  </si>
+  <si>
+    <t>Contabilización</t>
+  </si>
+  <si>
+    <t>Sistema deberá generar su debido asiento contable usando las cuentas del ramo de fianzas</t>
+  </si>
+  <si>
+    <t>Endosos</t>
+  </si>
+  <si>
+    <t>Cobros</t>
+  </si>
+  <si>
+    <t>Reservas</t>
+  </si>
+  <si>
+    <t>Pagos</t>
   </si>
 </sst>
 </file>
@@ -422,7 +441,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -454,6 +473,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2013,4 +2036,184 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E6FBF0A4-BF8A-48FC-893B-7F09853385EE}">
+  <sheetPr>
+    <tabColor rgb="FFFF0000"/>
+  </sheetPr>
+  <dimension ref="A1:H6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="16.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="4.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="5.5703125" style="12" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.85546875" style="12" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="7" style="12" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.28515625" style="12" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="82.7109375" style="12" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="11.42578125" style="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>98</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G2" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>100</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H3" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H4" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>17</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>